<commit_message>
Actualiza precios a mercado 2026 con fuentes y agrega guia PASO A PASO detallada
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/PRESUPUESTO CDI TESALIA - MODULO 1 (obra gris).xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/PRESUPUESTO CDI TESALIA - MODULO 1 (obra gris).xlsx
@@ -815,7 +815,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Precios de referencia COP - 2025. Fuente: Construdata 2025, listas de precios oficiales de obra (Gobernaciones) y cotizaciones tipicas. Validar con cotizaciones vigentes.</t>
+          <t>Precios de referencia COP - 2026. Fuente: cotizaciones de referencia (Argos, Homecenter, ferreterias y proveedores Huila), Construdata 2026 y SMLMV 2026 (Decreto 1469 de 2025). Reemplazar por cotizaciones formales si la entidad lo exige.</t>
         </is>
       </c>
     </row>
@@ -873,11 +873,11 @@
         </is>
       </c>
       <c r="E4" s="16" t="n">
-        <v>32000</v>
+        <v>34000</v>
       </c>
       <c r="F4" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. Homecenter/Argos 2026</t>
         </is>
       </c>
     </row>
@@ -903,11 +903,11 @@
         </is>
       </c>
       <c r="E5" s="16" t="n">
-        <v>78000</v>
+        <v>82000</v>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. proveedor agregados Neiva-Huila 2026</t>
         </is>
       </c>
     </row>
@@ -933,11 +933,11 @@
         </is>
       </c>
       <c r="E6" s="16" t="n">
-        <v>70000</v>
+        <v>74000</v>
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. proveedor agregados Neiva-Huila 2026</t>
         </is>
       </c>
     </row>
@@ -963,11 +963,11 @@
         </is>
       </c>
       <c r="E7" s="16" t="n">
-        <v>85000</v>
+        <v>88000</v>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. proveedor agregados Neiva-Huila 2026</t>
         </is>
       </c>
     </row>
@@ -993,11 +993,11 @@
         </is>
       </c>
       <c r="E8" s="16" t="n">
-        <v>8000</v>
+        <v>8500</v>
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Tarifa acueducto / carrotanque 2026</t>
         </is>
       </c>
     </row>
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="E9" s="16" t="n">
-        <v>560000</v>
+        <v>590000</v>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. Cementos Argos / Concretodo 2026</t>
         </is>
       </c>
     </row>
@@ -1053,11 +1053,11 @@
         </is>
       </c>
       <c r="E10" s="16" t="n">
-        <v>410000</v>
+        <v>430000</v>
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. Cementos Argos 2026</t>
         </is>
       </c>
     </row>
@@ -1083,11 +1083,11 @@
         </is>
       </c>
       <c r="E11" s="16" t="n">
-        <v>4600</v>
+        <v>4800</v>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. ferreteria/figurado (varilla 1/2") 2026</t>
         </is>
       </c>
     </row>
@@ -1113,11 +1113,11 @@
         </is>
       </c>
       <c r="E12" s="16" t="n">
-        <v>6800</v>
+        <v>7000</v>
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. ferreteria 2026</t>
         </is>
       </c>
     </row>
@@ -1143,11 +1143,11 @@
         </is>
       </c>
       <c r="E13" s="16" t="n">
-        <v>6200</v>
+        <v>6500</v>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. Acesco/ferreteria 2026</t>
         </is>
       </c>
     </row>
@@ -1173,11 +1173,11 @@
         </is>
       </c>
       <c r="E14" s="16" t="n">
-        <v>2500</v>
+        <v>2700</v>
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. bloquera local Huila 2026</t>
         </is>
       </c>
     </row>
@@ -1203,11 +1203,11 @@
         </is>
       </c>
       <c r="E15" s="16" t="n">
-        <v>2900</v>
+        <v>3100</v>
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. bloquera local Huila 2026</t>
         </is>
       </c>
     </row>
@@ -1233,11 +1233,11 @@
         </is>
       </c>
       <c r="E16" s="16" t="n">
-        <v>1250</v>
+        <v>1350</v>
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. prefabricados de concreto 2026</t>
         </is>
       </c>
     </row>
@@ -1263,11 +1263,11 @@
         </is>
       </c>
       <c r="E17" s="16" t="n">
-        <v>4200</v>
+        <v>4500</v>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. Pavco/Geomatrix 2026</t>
         </is>
       </c>
     </row>
@@ -1293,11 +1293,11 @@
         </is>
       </c>
       <c r="E18" s="16" t="n">
-        <v>92000</v>
+        <v>95000</v>
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. cantera/proveedor Huila 2026</t>
         </is>
       </c>
     </row>
@@ -1323,11 +1323,11 @@
         </is>
       </c>
       <c r="E19" s="16" t="n">
-        <v>62000</v>
+        <v>65000</v>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. cantera/proveedor Huila 2026</t>
         </is>
       </c>
     </row>
@@ -1353,11 +1353,11 @@
         </is>
       </c>
       <c r="E20" s="16" t="n">
-        <v>14000</v>
+        <v>15000</v>
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Construdata 2026 (costo por uso)</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Curador / antisol</t>
+          <t>Curador / antisol / impermeabilizante</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
@@ -1383,11 +1383,11 @@
         </is>
       </c>
       <c r="E21" s="16" t="n">
-        <v>45000</v>
+        <v>48000</v>
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. Sika/Toxement 2026</t>
         </is>
       </c>
     </row>
@@ -1413,11 +1413,11 @@
         </is>
       </c>
       <c r="E22" s="16" t="n">
-        <v>38000</v>
+        <v>40000</v>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. ferreteria 2026</t>
         </is>
       </c>
     </row>
@@ -1443,11 +1443,11 @@
         </is>
       </c>
       <c r="E23" s="16" t="n">
-        <v>70000</v>
+        <v>74000</v>
       </c>
       <c r="F23" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Cot. ref. proveedor agregados 2026</t>
         </is>
       </c>
     </row>
@@ -1473,11 +1473,11 @@
         </is>
       </c>
       <c r="E24" s="16" t="n">
-        <v>18000</v>
+        <v>19000</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>Construdata 2025</t>
+          <t>Construdata 2026</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="F25" s="17" t="inlineStr">
         <is>
-          <t>Resol. salarial 2025 + factor prestacional</t>
+          <t>SMLMV 2026 $1.750.905 (Dec.1469/25) x ~1.4 SMLMV + factor prestacional 1.55</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>Resol. salarial 2025 + factor prestacional</t>
+          <t>SMLMV 2026 $1.750.905 + aux. transporte + factor prestacional 1.55</t>
         </is>
       </c>
     </row>
@@ -1563,11 +1563,11 @@
         </is>
       </c>
       <c r="E27" s="16" t="n">
-        <v>150000</v>
+        <v>155000</v>
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>Tarifa alquiler equipo 2025</t>
+          <t>Tarifa alquiler maquinaria 2026</t>
         </is>
       </c>
     </row>
@@ -1593,11 +1593,11 @@
         </is>
       </c>
       <c r="E28" s="16" t="n">
-        <v>28000</v>
+        <v>30000</v>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>Tarifa alquiler equipo 2025</t>
+          <t>Tarifa transporte/disposicion 2026</t>
         </is>
       </c>
     </row>
@@ -1623,11 +1623,11 @@
         </is>
       </c>
       <c r="E29" s="16" t="n">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t>Tarifa alquiler equipo 2025</t>
+          <t>Tarifa alquiler equipo 2026</t>
         </is>
       </c>
     </row>
@@ -1653,11 +1653,11 @@
         </is>
       </c>
       <c r="E30" s="16" t="n">
-        <v>55000</v>
+        <v>58000</v>
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
-          <t>Tarifa alquiler equipo 2025</t>
+          <t>Tarifa alquiler equipo 2026</t>
         </is>
       </c>
     </row>
@@ -1683,11 +1683,11 @@
         </is>
       </c>
       <c r="E31" s="16" t="n">
-        <v>60000</v>
+        <v>62000</v>
       </c>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>Tarifa alquiler equipo 2025</t>
+          <t>Tarifa alquiler equipo 2026</t>
         </is>
       </c>
     </row>
@@ -1713,11 +1713,11 @@
         </is>
       </c>
       <c r="E32" s="16" t="n">
-        <v>50000</v>
+        <v>52000</v>
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
-          <t>Tarifa alquiler equipo 2025</t>
+          <t>Tarifa alquiler equipo 2026</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Curador / antisol  [Curador]</t>
+          <t>Curador / antisol / impermeabilizante  [Curador]</t>
         </is>
       </c>
       <c r="C48" s="15" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>Curador / antisol  [Curador]</t>
+          <t>Curador / antisol / impermeabilizante  [Curador]</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="B177" s="14" t="inlineStr">
         <is>
-          <t>Curador / antisol  [Impermeabilizante integral (gal)]</t>
+          <t>Curador / antisol / impermeabilizante  [Impermeabilizante integral (gal)]</t>
         </is>
       </c>
       <c r="C177" s="15" t="inlineStr">

</xml_diff>